<commit_message>
supabase table column changed and added new field
</commit_message>
<xml_diff>
--- a/src/AI/ML/SUPERVISED Learning/ds/supervised_excercise.xlsx
+++ b/src/AI/ML/SUPERVISED Learning/ds/supervised_excercise.xlsx
@@ -8,13 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Socourse\DE1\iot_api_dk\iot-data-engineering-platform\src\AI\ML\SUPERVISED Learning\ds\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED4A5A31-5E29-499D-91B9-D5292AB59FA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4576F019-FD7E-4156-9C0E-AC4B525D337E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" firstSheet="2" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Linear_Regression_Metrics_Workb" sheetId="1" r:id="rId1"/>
     <sheet name="Naive bayes metricseorkb" sheetId="2" r:id="rId2"/>
+    <sheet name="KNNxa" sheetId="3" r:id="rId3"/>
+    <sheet name="SVN" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -32,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="83">
   <si>
     <t>Salary(y)</t>
   </si>
@@ -248,6 +250,39 @@
   </si>
   <si>
     <t>Word frequency counts</t>
+  </si>
+  <si>
+    <t>X1</t>
+  </si>
+  <si>
+    <t>Y1</t>
+  </si>
+  <si>
+    <t>Euclidean Dist</t>
+  </si>
+  <si>
+    <t xml:space="preserve">class </t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>B</t>
+  </si>
+  <si>
+    <t>?</t>
+  </si>
+  <si>
+    <t>Predection</t>
+  </si>
+  <si>
+    <t>k = 1</t>
+  </si>
+  <si>
+    <t>nearest distance</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
   </si>
 </sst>
 </file>
@@ -1678,4 +1713,100 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB55FBB3-4018-4E6B-AF65-2CA5A4F5DCA1}">
+  <dimension ref="A1:F4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="3" max="3" width="11.77734375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>72</v>
+      </c>
+      <c r="B1" t="s">
+        <v>73</v>
+      </c>
+      <c r="C1" t="s">
+        <v>74</v>
+      </c>
+      <c r="D1" t="s">
+        <v>75</v>
+      </c>
+      <c r="E1" t="s">
+        <v>79</v>
+      </c>
+      <c r="F1" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>100</v>
+      </c>
+      <c r="B2">
+        <v>10</v>
+      </c>
+      <c r="C2">
+        <f>SQRT(SUM((A2-A3)^2)+(B2-B3)^2)</f>
+        <v>100.4987562112089</v>
+      </c>
+      <c r="D2" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>200</v>
+      </c>
+      <c r="B3">
+        <v>20</v>
+      </c>
+      <c r="C3">
+        <f t="shared" ref="C3:C4" si="0">SQRT(SUM((A3-A4)^2)+(B3-B4)^2)</f>
+        <v>100.4987562112089</v>
+      </c>
+      <c r="D3" t="s">
+        <v>78</v>
+      </c>
+      <c r="E3" t="s">
+        <v>76</v>
+      </c>
+      <c r="F3" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>300</v>
+      </c>
+      <c r="B4">
+        <v>30</v>
+      </c>
+      <c r="C4">
+        <f t="shared" si="0"/>
+        <v>301.4962686336267</v>
+      </c>
+      <c r="D4" t="s">
+        <v>77</v>
+      </c>
+      <c r="F4" t="s">
+        <v>82</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{08ABB480-4E42-433D-85C0-3FC8EEC6383B}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>